<commit_message>
Rebuild Mode 4 Golden Path doc with fresh Playwright run on mbx-ee-dev
Confirmed the BOQ -> Sold-as-Project -> Milestone -> Down Payment billing
overlay is unaffected by yesterday's Factory Worklist teardown (separate
mechanism). Re-verified both real bugs from the original build are still
fixed: BOQ-quoted price survives Select Lot Stock's quantity correction,
and delivery pulls from Stone Available rather than the never-populated
Stone Hold bucket. Fresh fixture: BOQ0029 -> SO S00126 -> Project 41 ->
INV/2026/00028-00030 -> EG01/OUT/00080. Also documented a real nuance: the
SO's own "Tasks" smart button only shows service-linked tasks (3 of 4) --
the Project's own Tasks view is needed to see the material line's task too.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client-docs/test-cases/emg-o-test-cases-e2e-mode4.xlsx
+++ b/client-docs/test-cases/emg-o-test-cases-e2e-mode4.xlsx
@@ -674,7 +674,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>สร้างใบเสนอราคาจากเอกสาร BOQ ("Generate Quotation")</t>
+          <t>สร้างใบเสนอราคาจากเอกสาร BOQ ("สร้างใบเสนอราคา")</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -691,14 +691,14 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>BOQ0026 — ลูกค้า "ทดสอบ Mode 4 Retest - Riverside Condo"
+          <t>BOQ0029 — ลูกค้า "ทดสอบ Mode4 Fresh - Sample Project"
 2 รายการ: Vietnam Limestone - Slab 0.5 ตร.ม. + Dry-Lay 1.5 ตร.ม.
 Preliminaries 5% + Overhead &amp; Profit 10%</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>สถานะ BOQ เปลี่ยนเป็น "Quotation Generated" เกิด Sale Order ใหม่ 1 ใบอัตโนมัติ ดึงทุกรายการ + ค่า Preliminaries/Overhead มาเป็นบรรทัดในใบเสนอราคาให้ครบ — ตัวอย่างจริง: BOQ0026 (รวม 1,380.00 บาท ก่อน VAT) → SO S00109</t>
+          <t>สถานะ BOQ เปลี่ยนเป็น "Quotation Generated" เกิด Sale Order ใหม่ 1 ใบอัตโนมัติ ดึงทุกรายการ + ค่า Preliminaries/Overhead มาเป็นบรรทัดในใบเสนอราคาให้ครบ — ตัวอย่างจริง: BOQ0029 (รวม 1,380.00 บาท ก่อน VAT) → SO S00126</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -876,7 +876,7 @@
         <is>
           <t>1. ที่บรรทัดสินค้าหิน กดลิงก์ "Select Lot Stock"
 2. เลือก Lot ของ Material นั้น
-3. กรอกจำนวนตร.ม.ที่จะขายจริง (ดูได้จากคำอธิบายท้ายชื่อสินค้าในบรรทัด)
+3. กรอกจำนวนตร.ม.ที่จะขายจริง
 4. กดยืนยัน</t>
         </is>
       </c>
@@ -888,7 +888,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>บรรทัดผูกกับ Lot ที่เลือกสำเร็จ จำนวนเปลี่ยนเป็น 0.5 ตร.ม. ตามที่กรอก ราคารวมของบรรทัดยังคงเท่าเดิมกับที่ BOQ ตั้งไว้เป๊ะ (ระบบคำนวณราคาต่อหน่วยใหม่ให้เอง) — ตัวอย่างจริง: ราคาต่อหน่วยเปลี่ยนจาก 900.00 (ที่จำนวน 1 หน่วยตั้งต้น) เป็น 1,800.00 บาท/ตร.ม. × 0.5 ตร.ม. = ยอดรวม 900.00 บาท เท่าเดิมทุกบาท</t>
+          <t>บรรทัดผูกกับ Lot ที่เลือกสำเร็จ จำนวนเปลี่ยนเป็น 0.5 ตร.ม. ตามที่กรอก ราคารวมของบรรทัดยังคงเท่าเดิมกับที่ BOQ ตั้งไว้เป๊ะ (ตัวอย่างจริง: ยอดรวม SO ยังคงเป็น 1,476.60 บาท เท่าเดิม ไม่เปลี่ยนหลังผูก Lot)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>✅ เคยพบปัญหาจริงตรงนี้ (ราคาที่ BOQ ตั้งไว้ถูกเขียนทับด้วยราคาป้ายสินค้าปกติ) — แก้ไขแล้วและทดสอบซ้ำผ่านในรอบนี้: ระบบคำนวณราคาต่อหน่วยใหม่ให้อัตโนมัติจากยอดรวมเดิมที่ BOQ ตั้งไว้ ไม่ใช้ราคาป้ายสินค้าอีกต่อไป</t>
+          <t>✅ ยืนยันแล้วว่าบั๊กเดิม (ราคาที่ BOQ ตั้งไว้ถูกเขียนทับด้วยราคาป้ายสินค้าปกติ) ยังคงปิดอยู่จริง: ระบบคำนวณราคาต่อหน่วยใหม่ให้อัตโนมัติจากยอดรวมเดิมที่ BOQ ตั้งไว้ ไม่ใช้ราคาป้ายสินค้า</t>
         </is>
       </c>
       <c r="I4" s="7" t="n"/>
@@ -934,7 +934,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>SO เปลี่ยนสถานะเป็น "Sales Order" เกิดปุ่ม/สถิติใหม่มุมบน: "Projects 1", "Tasks", "Delivery 1", "Invoices" — ไม่ต้องสร้าง Project เองแยกต่างหาก — ตัวอย่างจริง: S00109 (ยอดรวม 1,476.60 บาท รวม VAT) → Project id 40</t>
+          <t>SO เปลี่ยนสถานะเป็น "Sales Order" เกิดปุ่ม/สถิติใหม่มุมบน: "Projects 1", "Tasks 3", "Delivery 1" — ไม่ต้องสร้าง Project เองแยกต่างหาก — ตัวอย่างจริง: S00126 (ยอดรวม 1,476.60 บาท รวม VAT) → Project id 41</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -966,7 +966,8 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>1. กดปุ่มสถิติ "Tasks" บน Sale Order (หรือเปิด Project แล้วดู Tasks)</t>
+          <t>1. เปิด Project ของ SO นี้ (กดปุ่มสถิติ "Projects" บน Sale Order)
+2. กดปุ่มสถิติ "Tasks" บน Project (ไม่ใช่บน Sale Order)</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -976,7 +977,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>เห็น Task ครบ 1 งานต่อ 1 บรรทัดสินค้า/บริการ — ตัวอย่างจริง: 4 Tasks ("Vietnam Limestone - Slab (ปูพื้นระเบียง)...", "Dry-Lay", "BOQ Summary Line Preliminaries (5%)", "BOQ Summary Line Overhead &amp; Profit (10%)")</t>
+          <t>เห็น Task ครบ 4 งาน หนึ่งงานต่อหนึ่งบรรทัดสินค้า/บริการ — ตัวอย่างจริง: "Vietnam Limestone - Slab (ปูพื้นระเบียง) — 0.5 m²", "Dry-Lay", "BOQ Summary Line Preliminaries (5%)", "BOQ Summary Line Overhead &amp; Profit (10%)"</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -986,7 +987,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>หมายเหตุ: แต่ละบรรทัดใน SO (รวมถึงบรรทัด Preliminaries/Overhead &amp; Profit ที่เป็นแค่ตัวเลขสรุป ไม่ใช่งานจริง) จะได้ Task ของตัวเอง 1 งานเสมอ — เป็นพฤติกรรมที่ทราบอยู่แล้ว (ยังไม่กรองออก) ไม่ใช่ error หากเห็น Task ชื่อ "BOQ Summary Line Preliminaries/Overhead &amp; Profit" ปนอยู่กับงานจริง</t>
+          <t>หมายเหตุ: ปุ่มสถิติ "Tasks" บน Sale Order เอง จะโชว์ให้เห็นแค่ Task ที่เป็นบรรทัดบริการ (3 จาก 4 งาน) เพราะบรรทัดสินค้าวัสดุจริงผูก sale_line_id ไม่ได้ตามข้อจำกัดของระบบ — ต้องเปิด Project เองแล้วดู Tasks จากตรงนั้นถึงจะเห็นครบทั้ง 4 งาน แต่ละบรรทัดใน SO (รวมถึงบรรทัด Preliminaries/Overhead &amp; Profit ที่เป็นแค่ตัวเลขสรุป ไม่ใช่งานจริง) จะได้ Task ของตัวเอง 1 งานเสมอ</t>
         </is>
       </c>
       <c r="I6" s="7" t="n"/>
@@ -1125,7 +1126,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้สถานะ Posted ยอด 30% ของยอดรวม SO — ตัวอย่างจริง: INV/2026/00015 (442.98 บาท จาก 1,476.60 × 30%)</t>
+          <t>ใบแจ้งหนี้สถานะ Posted ยอด 30% ของยอดรวม SO — ตัวอย่างจริง: INV/2026/00028 (442.98 บาท จาก 1,476.60 × 30%)</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1170,7 +1171,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้สถานะ Posted ยอด 40% ของยอดรวม SO — ตัวอย่างจริง: INV/2026/00016 (590.64 บาท จาก 1,476.60 × 40%)</t>
+          <t>ใบแจ้งหนี้สถานะ Posted ยอด 40% ของยอดรวม SO — ตัวอย่างจริง: INV/2026/00029 (590.64 บาท จาก 1,476.60 × 40%)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1215,7 +1216,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้สถานะ Posted ยอดงวดสุดท้าย รวม 3 ใบแล้วเท่ากับยอด SO เป๊ะ — ตัวอย่างจริง: INV/2026/00017 (442.98 บาท) รวม 3 ใบ = 442.98 + 590.64 + 442.98 = 1,476.60 บาท ตรงกับยอด SO พอดี</t>
+          <t>ใบแจ้งหนี้สถานะ Posted ยอดงวดสุดท้าย รวม 3 ใบแล้วเท่ากับยอด SO เป๊ะ — ตัวอย่างจริง: INV/2026/00030 (442.98 บาท) รวม 3 ใบ = 442.98 + 590.64 + 442.98 = 1,476.60 บาท ตรงกับยอด SO พอดี</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1347,19 +1348,19 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>1. เปิด Inventory &gt; Deliveries
-2. เปิดใบส่งของของ SO นี้
+          <t>1. เปิด Sale Order &gt; กดปุ่มสถิติ "Delivery"
+2. กด "Details" ที่บรรทัดสินค้า กรอกช่อง "Scanned Serial" ให้ตรงกับชื่อ Lot แล้ว Save
 3. กด Validate</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Scanned Serial = BLK-26-0004-LOT</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ใบส่งของเปลี่ยนสถานะเป็น Done ดึงสต็อกจากจุดที่ของจริงอยู่ถูกต้อง — ตัวอย่างจริง: EG01/OUT/00064 (Vietnam Limestone - Slab 0.5 ตร.ม., Pick From "Stone Inventory/Stone Available")</t>
+          <t>ใบส่งของเปลี่ยนสถานะเป็น Done ดึงสต็อกจากจุดที่ของจริงอยู่ถูกต้อง — ตัวอย่างจริง: EG01/OUT/00080 (Vietnam Limestone - Slab 0.5 ตร.ม., Source Location "EG01/Stock")</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1369,7 +1370,7 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>✅ เคยพบปัญหาจริงตรงนี้ (ระบบดึงสต็อกจากจุดพัก "Stone Hold" ที่โหมด Lot ไม่เคยย้ายของเข้าจริง ทำให้ยอดติดลบเพิ่มขึ้นทุกครั้งที่ส่งของ) — แก้ไขแล้วและทดสอบซ้ำผ่านในรอบนี้: ระบบดึงสต็อกจากจุดที่ของจริงอยู่ ("Stone Available") แทน ดูรายละเอียดที่ปุ่ม "Details" ในรายการส่งของ</t>
+          <t>✅ ยืนยันแล้วว่าบั๊กเดิม (ระบบดึงสต็อกจากจุดพัก "Stone Hold" ที่โหมด Lot ไม่เคยย้ายของเข้าจริง ทำให้ยอดติดลบเพิ่มขึ้นทุกครั้งที่ส่งของ) ยังคงปิดอยู่จริง: ระบบดึงสต็อกจากจุดที่ของจริงอยู่ ("Stone Available") ถูกต้อง — ต้องกรอก Scanned Serial ให้ตรงกับชื่อ Lot ก่อน Validate เสมอ (ตรรกะเดียวกับ Mode 2/3)</t>
         </is>
       </c>
       <c r="I4" s="7" t="n"/>
@@ -1496,7 +1497,7 @@
       <c r="D4" s="7" t="inlineStr">
         <is>
           <t>1. เปิด Task "Dry-Lay"
-2. เลื่อนสถานะ Task ไปช่อง/สถานะ Done</t>
+2. กดป้ายสถานะมุมขวาบน (เช่น "In Progress") เลือก "Done"</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -1506,7 +1507,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>Task ขึ้นเครื่องหมายเสร็จ และ Milestone ที่ผูกกับ Task นั้นเปลี่ยนเป็น "Reached" ให้อัตโนมัติ โดยไม่ต้องไปกดยืนยัน Milestone แยกต่างหาก — ตัวอย่างจริง: Milestone "ปูพื้นระเบียงเสร็จสมบูรณ์ (Dry-Lay Complete)" ขึ้นเครื่องหมายถูกในหน้า Project Dashboard ทันที</t>
+          <t>Task ขึ้นป้ายสถานะ "Done" และ Milestone ที่ผูกกับ Task นั้นเปลี่ยนเป็นติ๊กถูกให้อัตโนมัติ โดยไม่ต้องไปกดยืนยัน Milestone แยกต่างหาก — ตัวอย่างจริง: Milestone "ปูพื้นเสร็จสมบูรณ์ (Dry-Lay Complete)" ขึ้นเครื่องหมายถูกในหน้า Project Dashboard ทันที</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1538,9 +1539,8 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>1. เปิด Project ของ SO นี้
-2. กดปุ่มสถิติ "Tasks"
-3. สลับมุมมองด้านขวาบนเป็น "Gantt"</t>
+          <t>1. เปิด Project ของ SO นี้ &gt; กดปุ่มสถิติ "Tasks"
+2. สลับมุมมองด้านขวาบนเป็น "Gantt"</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -1550,7 +1550,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>เห็นแท่ง Gantt ของแต่ละ Task เรียงตามวันที่วางแผน (จากช่อง Duration ที่กรอกไว้ตอนสร้าง BOQ) กลุ่มตามผู้รับผิดชอบ — Task ที่ทำเสร็จแล้วแสดงเป็นแท่งสีเทาจาง</t>
+          <t>เห็นแท่ง Gantt ของแต่ละ Task เรียงตามวันที่วางแผน กลุ่มตามผู้รับผิดชอบ — Task ที่ทำเสร็จแล้ว (Dry-Lay) จะหายไปจากมุมมองนี้เพราะ filter เริ่มต้นกรองเฉพาะงานที่ยังเปิดอยู่ ("Open") — ปิด filter นี้ถ้าต้องการเห็นงานที่เสร็จแล้วด้วย</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1683,7 +1683,7 @@
       <c r="D4" s="7" t="inlineStr">
         <is>
           <t>1. เปิด Project ของ SO นี้
-2. ดูส่วน "Profitability" บนหน้า Dashboard ของ Project</t>
+2. กดปุ่มสถิติ "Dashboard"</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>เดบิต/เครดิตสมดุลกัน (รวมเท่ากันทั้ง 2 ฝั่ง) เห็น Analytic Distribution ผูกกับบัญชี Analytic ของโปรเจกต์นี้บนบรรทัดรายได้ — ตัวอย่างจริง: INV/2026/00017 เดบิต Trade Receivables 442.98 = เครดิต Down Payment 414.00 + Output VAT 28.98 พอดี พร้อมป้าย Analytic "BOQ0026 - ทดสอบ Mode 4 Retest..."</t>
+          <t>เดบิต/เครดิตสมดุลกัน (รวมเท่ากันทั้ง 2 ฝั่ง) เห็น Analytic Distribution ผูกกับบัญชี Analytic ของโปรเจกต์นี้บนบรรทัดรายได้ — ตัวอย่างจริง: INV/2026/00030 เดบิต Trade Receivables 442.98 = เครดิต Down Payment 414.00 + Output VAT 28.98 พอดี พร้อมป้าย Analytic "BOQ0029 - ทดสอบ Mode4 Fresh..."</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">

</xml_diff>